<commit_message>
Fix admin notification and A4 delivery export
</commit_message>
<xml_diff>
--- a/outputs/delivery-note-template/Chaphranakhon_Delivery_Note_Template_A4.xlsx
+++ b/outputs/delivery-note-template/Chaphranakhon_Delivery_Note_Template_A4.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Delivery Note" sheetId="1" ns1:id="Rea8b0e9969754d8f"/>
+    <sheet name="Delivery Note" sheetId="1" ns1:id="Re44e6e9354ff4bf0"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Delivery Note'!$A$1:$J$60</definedName>
@@ -648,13 +648,13 @@
     <xdr:ext cx="1619250" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1c4d6eb7-af03-4fbe-8856-9dc1bea5cd0e"/>
+        <xdr:cNvPr id="1" name="61a08d4e-70d8-4455-9565-e9a861b66bf8"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R64dda25301834b8a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R62e62839fa2e498d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1010,7 +1010,7 @@
       <c r="I10" s="15"/>
       <c r="J10" s="16"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="3" customHeight="1">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1022,7 +1022,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="3" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1034,7 +1034,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="3" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1160,7 +1160,7 @@
         <v>จำนวนเงิน</v>
       </c>
     </row>
-    <row r="21" ht="4" customHeight="1">
+    <row r="21" ht="3" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1817,6 +1817,6 @@
   <printOptions horizontalCentered="1" verticalCentered="0"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="1" blackAndWhite="0" draft="0"/>
-  <drawing ns1:id="Rdac88f6088c14376"/>
+  <drawing ns1:id="Rc82ee35f4d6c4fd3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add document templates and previews
</commit_message>
<xml_diff>
--- a/outputs/delivery-note-template/Chaphranakhon_Delivery_Note_Template_A4.xlsx
+++ b/outputs/delivery-note-template/Chaphranakhon_Delivery_Note_Template_A4.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Delivery Note" sheetId="1" ns1:id="Re44e6e9354ff4bf0"/>
+    <sheet name="Delivery Note" sheetId="1" ns1:id="Rd9aeff8e427e4b20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Delivery Note'!$A$1:$J$60</definedName>
@@ -401,16 +401,13 @@
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -548,79 +545,82 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -648,13 +648,13 @@
     <xdr:ext cx="1619250" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="61a08d4e-70d8-4455-9565-e9a861b66bf8"/>
+        <xdr:cNvPr id="1" name="d8ee596d-2f6f-48a9-9046-c391cc02ca06"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R62e62839fa2e498d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4cfd55728d934287"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1172,426 +1172,426 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="17" customHeight="1">
       <c r="A22" s="2"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35" t="str">
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34" t="str">
         <f>IF(OR(G22="",I22=""),"",G22*I22)</f>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="17" customHeight="1">
       <c r="A23" s="2"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35" t="str">
+      <c r="B23" s="32"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="34"/>
+      <c r="J23" s="34" t="str">
         <f>IF(OR(G23="",I23=""),"",G23*I23)</f>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="17" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35" t="str">
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="34"/>
+      <c r="J24" s="34" t="str">
         <f>IF(OR(G24="",I24=""),"",G24*I24)</f>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25" ht="17" customHeight="1">
       <c r="A25" s="2"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="35" t="str">
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="34" t="str">
         <f>IF(OR(G25="",I25=""),"",G25*I25)</f>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="17" customHeight="1">
       <c r="A26" s="2"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35" t="str">
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34" t="str">
         <f>IF(OR(G26="",I26=""),"",G26*I26)</f>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
+    <row r="27" ht="17" customHeight="1">
       <c r="A27" s="2"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="35" t="str">
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="34"/>
+      <c r="J27" s="34" t="str">
         <f>IF(OR(G27="",I27=""),"",G27*I27)</f>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28" ht="17" customHeight="1">
       <c r="A28" s="2"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="35"/>
-      <c r="J28" s="35" t="str">
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34" t="str">
         <f>IF(OR(G28="",I28=""),"",G28*I28)</f>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="17" customHeight="1">
       <c r="A29" s="2"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35" t="str">
+      <c r="B29" s="32"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34" t="str">
         <f>IF(OR(G29="",I29=""),"",G29*I29)</f>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" ht="17" customHeight="1">
       <c r="A30" s="2"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="33"/>
-      <c r="D30" s="33"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="35"/>
-      <c r="J30" s="35" t="str">
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34" t="str">
         <f>IF(OR(G30="",I30=""),"",G30*I30)</f>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="17" customHeight="1">
       <c r="A31" s="2"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35" t="str">
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34" t="str">
         <f>IF(OR(G31="",I31=""),"",G31*I31)</f>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32" ht="17" customHeight="1">
       <c r="A32" s="2"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="33"/>
-      <c r="D32" s="33"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="35"/>
-      <c r="J32" s="35" t="str">
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="34"/>
+      <c r="J32" s="34" t="str">
         <f>IF(OR(G32="",I32=""),"",G32*I32)</f>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33" ht="17" customHeight="1">
       <c r="A33" s="2"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="35" t="str">
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="34"/>
+      <c r="J33" s="34" t="str">
         <f>IF(OR(G33="",I33=""),"",G33*I33)</f>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1">
+    <row r="34" ht="17" customHeight="1">
       <c r="A34" s="2"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="33"/>
-      <c r="I34" s="35"/>
-      <c r="J34" s="35" t="str">
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="34" t="str">
         <f>IF(OR(G34="",I34=""),"",G34*I34)</f>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
+    <row r="35" ht="17" customHeight="1">
       <c r="A35" s="2"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="33"/>
-      <c r="I35" s="35"/>
-      <c r="J35" s="35" t="str">
+      <c r="B35" s="32"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="34"/>
+      <c r="J35" s="34" t="str">
         <f>IF(OR(G35="",I35=""),"",G35*I35)</f>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1">
+    <row r="36" ht="17" customHeight="1">
       <c r="A36" s="2"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="35"/>
-      <c r="J36" s="35" t="str">
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="34" t="str">
         <f>IF(OR(G36="",I36=""),"",G36*I36)</f>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37" ht="17" customHeight="1">
       <c r="A37" s="2"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="33"/>
-      <c r="H37" s="33"/>
-      <c r="I37" s="35"/>
-      <c r="J37" s="35" t="str">
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="34"/>
+      <c r="J37" s="34" t="str">
         <f>IF(OR(G37="",I37=""),"",G37*I37)</f>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38" ht="17" customHeight="1">
       <c r="A38" s="2"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="33"/>
-      <c r="D38" s="33"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="33"/>
-      <c r="I38" s="35"/>
-      <c r="J38" s="35" t="str">
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="34"/>
+      <c r="J38" s="34" t="str">
         <f>IF(OR(G38="",I38=""),"",G38*I38)</f>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
+    <row r="39" ht="17" customHeight="1">
       <c r="A39" s="2"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="33"/>
-      <c r="I39" s="35"/>
-      <c r="J39" s="35" t="str">
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="34"/>
+      <c r="J39" s="34" t="str">
         <f>IF(OR(G39="",I39=""),"",G39*I39)</f>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1">
+    <row r="40" ht="17" customHeight="1">
       <c r="A40" s="2"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="33"/>
-      <c r="H40" s="33"/>
-      <c r="I40" s="35"/>
-      <c r="J40" s="35" t="str">
+      <c r="B40" s="32"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="34"/>
+      <c r="J40" s="34" t="str">
         <f>IF(OR(G40="",I40=""),"",G40*I40)</f>
       </c>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41" ht="17" customHeight="1">
       <c r="A41" s="2"/>
-      <c r="B41" s="33"/>
-      <c r="C41" s="33"/>
-      <c r="D41" s="33"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="33"/>
-      <c r="H41" s="33"/>
-      <c r="I41" s="35"/>
-      <c r="J41" s="35" t="str">
+      <c r="B41" s="32"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="34"/>
+      <c r="J41" s="34" t="str">
         <f>IF(OR(G41="",I41=""),"",G41*I41)</f>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42" ht="17" customHeight="1">
       <c r="A42" s="2"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="33"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="33"/>
-      <c r="I42" s="35"/>
-      <c r="J42" s="35" t="str">
+      <c r="B42" s="32"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="34"/>
+      <c r="J42" s="34" t="str">
         <f>IF(OR(G42="",I42=""),"",G42*I42)</f>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43" ht="17" customHeight="1">
       <c r="A43" s="2"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="33"/>
-      <c r="H43" s="33"/>
-      <c r="I43" s="35"/>
-      <c r="J43" s="35" t="str">
+      <c r="B43" s="32"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="34"/>
+      <c r="J43" s="34" t="str">
         <f>IF(OR(G43="",I43=""),"",G43*I43)</f>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44" ht="17" customHeight="1">
       <c r="A44" s="2"/>
-      <c r="B44" s="33"/>
-      <c r="C44" s="33"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="33"/>
-      <c r="I44" s="35"/>
-      <c r="J44" s="35" t="str">
+      <c r="B44" s="32"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="34"/>
+      <c r="J44" s="34" t="str">
         <f>IF(OR(G44="",I44=""),"",G44*I44)</f>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="17" customHeight="1">
       <c r="A45" s="2"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="33"/>
-      <c r="D45" s="33"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="33"/>
-      <c r="H45" s="33"/>
-      <c r="I45" s="35"/>
-      <c r="J45" s="35" t="str">
+      <c r="B45" s="32"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="34"/>
+      <c r="J45" s="34" t="str">
         <f>IF(OR(G45="",I45=""),"",G45*I45)</f>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2"/>
-      <c r="B46" s="69" t="str">
+      <c r="B46" s="68" t="str">
         <v>หมายเหตุ
 เอกสารนี้เป็นใบส่งของและแสดง VAT เพื่อให้ผู้ซื้อทราบยอดที่ต้องชำระจริง
 ค่าขนส่งและค่าใช้จ่ายอื่นไม่รวมอยู่ในฐานคำนวณ VAT</v>
       </c>
-      <c r="C46" s="70"/>
-      <c r="D46" s="70"/>
-      <c r="E46" s="70"/>
-      <c r="F46" s="70"/>
-      <c r="G46" s="71"/>
-      <c r="H46" s="39" t="str">
+      <c r="C46" s="69"/>
+      <c r="D46" s="69"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="69"/>
+      <c r="G46" s="70"/>
+      <c r="H46" s="38" t="str">
         <v>ค่าวัตถุดิบรวม</v>
       </c>
-      <c r="I46" s="39"/>
-      <c r="J46" s="41" t="n">
+      <c r="I46" s="38"/>
+      <c r="J46" s="40" t="n">
         <f>SUM(J22:J45)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="2"/>
-      <c r="B47" s="72"/>
-      <c r="C47" s="73"/>
-      <c r="D47" s="73"/>
-      <c r="E47" s="73"/>
-      <c r="F47" s="73"/>
-      <c r="G47" s="74"/>
-      <c r="H47" s="39" t="str">
+      <c r="B47" s="71"/>
+      <c r="C47" s="72"/>
+      <c r="D47" s="72"/>
+      <c r="E47" s="72"/>
+      <c r="F47" s="72"/>
+      <c r="G47" s="73"/>
+      <c r="H47" s="38" t="str">
         <v>ส่วนลด</v>
       </c>
-      <c r="I47" s="39"/>
-      <c r="J47" s="41" t="n">
+      <c r="I47" s="38"/>
+      <c r="J47" s="40" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2"/>
-      <c r="B48" s="72"/>
-      <c r="C48" s="73"/>
-      <c r="D48" s="73"/>
-      <c r="E48" s="73"/>
-      <c r="F48" s="73"/>
-      <c r="G48" s="74"/>
-      <c r="H48" s="39" t="str">
+      <c r="B48" s="71"/>
+      <c r="C48" s="72"/>
+      <c r="D48" s="72"/>
+      <c r="E48" s="72"/>
+      <c r="F48" s="72"/>
+      <c r="G48" s="73"/>
+      <c r="H48" s="38" t="str">
         <v>ยอดก่อน VAT</v>
       </c>
-      <c r="I48" s="39"/>
-      <c r="J48" s="41" t="n">
+      <c r="I48" s="38"/>
+      <c r="J48" s="40" t="n">
         <f>MAX(0,J46-J47)</f>
         <v>0</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="2"/>
-      <c r="B49" s="72"/>
-      <c r="C49" s="73"/>
-      <c r="D49" s="73"/>
-      <c r="E49" s="73"/>
-      <c r="F49" s="73"/>
-      <c r="G49" s="74"/>
-      <c r="H49" s="39" t="str">
+      <c r="B49" s="71"/>
+      <c r="C49" s="72"/>
+      <c r="D49" s="72"/>
+      <c r="E49" s="72"/>
+      <c r="F49" s="72"/>
+      <c r="G49" s="73"/>
+      <c r="H49" s="38" t="str">
         <v>VAT 7%</v>
       </c>
-      <c r="I49" s="39"/>
-      <c r="J49" s="41" t="n">
+      <c r="I49" s="38"/>
+      <c r="J49" s="40" t="n">
         <f>ROUND(J48*7%,2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="2"/>
-      <c r="B50" s="75"/>
-      <c r="C50" s="76"/>
-      <c r="D50" s="76"/>
-      <c r="E50" s="76"/>
-      <c r="F50" s="76"/>
-      <c r="G50" s="77"/>
-      <c r="H50" s="39" t="str">
+      <c r="B50" s="74"/>
+      <c r="C50" s="75"/>
+      <c r="D50" s="75"/>
+      <c r="E50" s="75"/>
+      <c r="F50" s="75"/>
+      <c r="G50" s="76"/>
+      <c r="H50" s="38" t="str">
         <v>ค่าขนส่ง / ค่าใช้จ่ายอื่น (ไม่คิด VAT)</v>
       </c>
-      <c r="I50" s="39"/>
-      <c r="J50" s="41" t="n">
+      <c r="I50" s="38"/>
+      <c r="J50" s="40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1615,28 +1615,28 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
-      <c r="H52" s="48" t="str">
+      <c r="H52" s="47" t="str">
         <v>ยอดรวมทั้งสิ้น</v>
       </c>
-      <c r="I52" s="49"/>
-      <c r="J52" s="50" t="n">
+      <c r="I52" s="48"/>
+      <c r="J52" s="49" t="n">
         <f>J48+J49+J50</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" ht="24" customHeight="1">
       <c r="A53" s="2"/>
-      <c r="B53" s="78" t="str">
+      <c r="B53" s="77" t="str">
         <v>ชำระโดย / Paid By     □ เงินสด     □ โอนเงิน ธนาคาร __________________________     □ เช็คธนาคาร __________________________</v>
       </c>
-      <c r="C53" s="79"/>
-      <c r="D53" s="79"/>
-      <c r="E53" s="79"/>
-      <c r="F53" s="79"/>
-      <c r="G53" s="79"/>
-      <c r="H53" s="79"/>
-      <c r="I53" s="79"/>
-      <c r="J53" s="80"/>
+      <c r="C53" s="78"/>
+      <c r="D53" s="78"/>
+      <c r="E53" s="78"/>
+      <c r="F53" s="78"/>
+      <c r="G53" s="78"/>
+      <c r="H53" s="78"/>
+      <c r="I53" s="78"/>
+      <c r="J53" s="79"/>
     </row>
     <row r="54" ht="4" customHeight="1">
       <c r="A54" s="2"/>
@@ -1817,6 +1817,6 @@
   <printOptions horizontalCentered="1" verticalCentered="0"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="1" blackAndWhite="0" draft="0"/>
-  <drawing ns1:id="Rc82ee35f4d6c4fd3"/>
+  <drawing ns1:id="R123ec04eb5a5470f"/>
 </worksheet>
 </file>
</xml_diff>